<commit_message>
Contents v002 (exposure fix + mode imputation, CV 4,858->63.6), Buildings v003 (mode imputation, monotonicity 78%->89%), combined v007/v008, new buildings/contents EDA notebooks + Excel
</commit_message>
<xml_diff>
--- a/Excel files/buildings_tweedie_xgb_results.xlsx
+++ b/Excel files/buildings_tweedie_xgb_results.xlsx
@@ -465,13 +465,13 @@
         <v>59619</v>
       </c>
       <c r="C2" t="n">
-        <v>16.51198815050339</v>
+        <v>17.03940151138826</v>
       </c>
       <c r="D2" t="n">
-        <v>82.26811066941747</v>
+        <v>88.69040138210973</v>
       </c>
       <c r="E2" t="n">
-        <v>0.01816534997232426</v>
+        <v>0.01798084503262383</v>
       </c>
     </row>
     <row r="3">
@@ -482,13 +482,13 @@
         <v>59619</v>
       </c>
       <c r="C3" t="n">
-        <v>29.49169543764464</v>
+        <v>30.26188251449484</v>
       </c>
       <c r="D3" t="n">
-        <v>118.1047359063386</v>
+        <v>126.0619423338198</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02210704641137892</v>
+        <v>0.0225599221724618</v>
       </c>
     </row>
     <row r="4">
@@ -499,13 +499,13 @@
         <v>59618</v>
       </c>
       <c r="C4" t="n">
-        <v>39.74442037351857</v>
+        <v>40.63905724458875</v>
       </c>
       <c r="D4" t="n">
-        <v>113.0602373444262</v>
+        <v>139.7419517595357</v>
       </c>
       <c r="E4" t="n">
-        <v>0.024170552517696</v>
+        <v>0.025562749505183</v>
       </c>
     </row>
     <row r="5">
@@ -513,16 +513,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>59620</v>
+        <v>59619</v>
       </c>
       <c r="C5" t="n">
-        <v>49.97799076226205</v>
+        <v>50.99074241341167</v>
       </c>
       <c r="D5" t="n">
-        <v>155.8196772895002</v>
+        <v>135.2016924134923</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0282120093928212</v>
+        <v>0.02728995789932739</v>
       </c>
     </row>
     <row r="6">
@@ -530,16 +530,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>59617</v>
+        <v>59618</v>
       </c>
       <c r="C6" t="n">
-        <v>61.10086879483556</v>
+        <v>62.1816722566325</v>
       </c>
       <c r="D6" t="n">
-        <v>173.8027851116292</v>
+        <v>148.3612989365628</v>
       </c>
       <c r="E6" t="n">
-        <v>0.03188687790395357</v>
+        <v>0.02987352812908853</v>
       </c>
     </row>
     <row r="7">
@@ -547,16 +547,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>59620</v>
+        <v>59619</v>
       </c>
       <c r="C7" t="n">
-        <v>73.98619889672352</v>
+        <v>75.17722426668685</v>
       </c>
       <c r="D7" t="n">
-        <v>168.5102428715196</v>
+        <v>181.6799352555394</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0316839986581684</v>
+        <v>0.03356312584914205</v>
       </c>
     </row>
     <row r="8">
@@ -564,16 +564,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>59617</v>
+        <v>59618</v>
       </c>
       <c r="C8" t="n">
-        <v>89.87511949471839</v>
+        <v>91.2868594016979</v>
       </c>
       <c r="D8" t="n">
-        <v>191.9796172232752</v>
+        <v>186.0484759636351</v>
       </c>
       <c r="E8" t="n">
-        <v>0.03584548031601725</v>
+        <v>0.03616357475930088</v>
       </c>
     </row>
     <row r="9">
@@ -584,13 +584,13 @@
         <v>59619</v>
       </c>
       <c r="C9" t="n">
-        <v>111.7538210851032</v>
+        <v>113.2671090071347</v>
       </c>
       <c r="D9" t="n">
-        <v>218.2585045035978</v>
+        <v>236.0706571730489</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0409936429661685</v>
+        <v>0.04079236485013167</v>
       </c>
     </row>
     <row r="10">
@@ -601,13 +601,13 @@
         <v>59618</v>
       </c>
       <c r="C10" t="n">
-        <v>146.7717489189893</v>
+        <v>148.5491141840406</v>
       </c>
       <c r="D10" t="n">
-        <v>267.3760090912141</v>
+        <v>241.6554842497232</v>
       </c>
       <c r="E10" t="n">
-        <v>0.04604314133315442</v>
+        <v>0.04592572712939045</v>
       </c>
     </row>
     <row r="11">
@@ -618,13 +618,13 @@
         <v>59619</v>
       </c>
       <c r="C11" t="n">
-        <v>265.1224559568371</v>
+        <v>265.5009873019295</v>
       </c>
       <c r="D11" t="n">
-        <v>374.1818876532649</v>
+        <v>379.8487628105134</v>
       </c>
       <c r="E11" t="n">
-        <v>0.05857193176671866</v>
+        <v>0.05796809741860817</v>
       </c>
     </row>
   </sheetData>
@@ -665,36 +665,36 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>75496.0302734375</v>
+        <v>68762.98828125</v>
       </c>
       <c r="C2" t="n">
-        <v>0.07340245111801089</v>
+        <v>0.06790626280944632</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>new_business</t>
+          <t>elevation_m</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>34602.60107421875</v>
+        <v>34351.5673828125</v>
       </c>
       <c r="C3" t="n">
-        <v>0.03364303692137328</v>
+        <v>0.0339235775076072</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>elevation_m</t>
+          <t>new_business</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>32421.31396484375</v>
+        <v>30166.41748046875</v>
       </c>
       <c r="C4" t="n">
-        <v>0.03152223904842102</v>
+        <v>0.02979057083833513</v>
       </c>
     </row>
     <row r="5">
@@ -704,10 +704,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>28372.3203125</v>
+        <v>27973.28076171875</v>
       </c>
       <c r="C5" t="n">
-        <v>0.02758552797146964</v>
+        <v>0.02762475864600646</v>
       </c>
     </row>
     <row r="6">
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>27620.4140625</v>
+        <v>26895.8984375</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0268544728211385</v>
+        <v>0.02656079954412142</v>
       </c>
     </row>
     <row r="7">
@@ -730,10 +730,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>27178.50634765625</v>
+        <v>26697.42724609375</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0264248196417593</v>
+        <v>0.02636480112664991</v>
       </c>
     </row>
     <row r="8">
@@ -743,75 +743,75 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26196.90234375</v>
+        <v>25759.376953125</v>
       </c>
       <c r="C8" t="n">
-        <v>0.02547043648210166</v>
+        <v>0.02543843810324153</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>trees_within_5m</t>
+          <t>occupation</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>25858.86669921875</v>
+        <v>25164.521484375</v>
       </c>
       <c r="C9" t="n">
-        <v>0.02514177489838684</v>
+        <v>0.02485099400279966</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>occupation</t>
+          <t>trees_within_5m</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>25606.02880859375</v>
+        <v>24764.783203125</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0248959484510867</v>
+        <v>0.0244562361038187</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>occupancy</t>
+          <t>missed_payments_12m</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>23149.94580078125</v>
+        <v>23481.4765625</v>
       </c>
       <c r="C11" t="n">
-        <v>0.02250797504016996</v>
+        <v>0.02318891831874868</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>bedrooms</t>
+          <t>region</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>23003.318359375</v>
+        <v>22906.58251953125</v>
       </c>
       <c r="C12" t="n">
-        <v>0.02236541372189402</v>
+        <v>0.02262118694253585</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>occupancy</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>22801.47119140625</v>
+        <v>22666.4384765625</v>
       </c>
       <c r="C13" t="n">
-        <v>0.02216916397437124</v>
+        <v>0.02238403488004461</v>
       </c>
     </row>
     <row r="14">
@@ -821,49 +821,49 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>22625.9287109375</v>
+        <v>22608.537109375</v>
       </c>
       <c r="C14" t="n">
-        <v>0.02199848945949842</v>
+        <v>0.0223268549122227</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>channel</t>
+          <t>bedrooms</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>22497.05810546875</v>
+        <v>22511.12109375</v>
       </c>
       <c r="C15" t="n">
-        <v>0.02187319256263898</v>
+        <v>0.02223065261322104</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>energy_rating</t>
+          <t>channel</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>21382.89599609375</v>
+        <v>21370.01171875</v>
       </c>
       <c r="C16" t="n">
-        <v>0.02078992726412285</v>
+        <v>0.02110376044273923</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>construction_type</t>
+          <t>smoke_alarms</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>21366.2783203125</v>
+        <v>21101.31689453125</v>
       </c>
       <c r="C17" t="n">
-        <v>0.02077377041283133</v>
+        <v>0.02083841331625445</v>
       </c>
     </row>
     <row r="18">
@@ -873,166 +873,166 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>21062.57861328125</v>
+        <v>21058.31982421875</v>
       </c>
       <c r="C18" t="n">
-        <v>0.02047849259730678</v>
+        <v>0.02079595195106865</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>basement</t>
+          <t>distance_to_river_km</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>20634.623046875</v>
+        <v>20984.7421875</v>
       </c>
       <c r="C19" t="n">
-        <v>0.02006240465956964</v>
+        <v>0.02072329102604478</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>distance_to_river_km</t>
+          <t>construction_type</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>19990.689453125</v>
+        <v>20583.69091796875</v>
       </c>
       <c r="C20" t="n">
-        <v>0.01943632797756018</v>
+        <v>0.02032723649744488</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>missed_payments_12m</t>
+          <t>energy_rating</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>19832.74536132812</v>
+        <v>20160.57958984375</v>
       </c>
       <c r="C21" t="n">
-        <v>0.01928276383073672</v>
+        <v>0.01990939675889552</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>dry_summer_index</t>
+          <t>basement</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>18863.4033203125</v>
+        <v>19848.39404296875</v>
       </c>
       <c r="C22" t="n">
-        <v>0.01834030259768144</v>
+        <v>0.01960110076534887</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>soil_type</t>
+          <t>accidental_damage_cover</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>18773.6328125</v>
+        <v>18698.5927734375</v>
       </c>
       <c r="C23" t="n">
-        <v>0.01825302151432275</v>
+        <v>0.01846562499358526</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>smoke_alarms</t>
+          <t>years_at_address</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>18662.1953125</v>
+        <v>18463.50732421875</v>
       </c>
       <c r="C24" t="n">
-        <v>0.01814467428577527</v>
+        <v>0.01823346849928005</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>solar_panels</t>
+          <t>hail_days</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>18531.33642578125</v>
+        <v>18337.6376953125</v>
       </c>
       <c r="C25" t="n">
-        <v>0.01801744424465999</v>
+        <v>0.01810916709362742</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>accidental_damage_cover</t>
+          <t>rainfall_mm</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>18497.3076171875</v>
+        <v>18259.78076171875</v>
       </c>
       <c r="C26" t="n">
-        <v>0.01798435908838938</v>
+        <v>0.01803228018794888</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>credit_band</t>
+          <t>dry_summer_index</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>18438.65478515625</v>
+        <v>18233.43603515625</v>
       </c>
       <c r="C27" t="n">
-        <v>0.01792733275706423</v>
+        <v>0.01800626369317005</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>hail_days</t>
+          <t>days_quote_to_inception</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>18395.81640625</v>
+        <v>18104.85107421875</v>
       </c>
       <c r="C28" t="n">
-        <v>0.01788568232852843</v>
+        <v>0.01787928078610018</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>years_at_address</t>
+          <t>property_type</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>18257.8740234375</v>
+        <v>17810.4033203125</v>
       </c>
       <c r="C29" t="n">
-        <v>0.01775156522363134</v>
+        <v>0.0175885015884506</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>rainfall_mm</t>
+          <t>marital_status</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>18233.39794921875</v>
+        <v>17801.13720703125</v>
       </c>
       <c r="C30" t="n">
-        <v>0.01772776789501822</v>
+        <v>0.01757935092267202</v>
       </c>
     </row>
     <row r="31">
@@ -1042,49 +1042,49 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>18188.1923828125</v>
+        <v>17788.79150390625</v>
       </c>
       <c r="C31" t="n">
-        <v>0.01768381592341947</v>
+        <v>0.01756715903599099</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>property_type</t>
+          <t>soil_type</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>18096.59326171875</v>
+        <v>17674.35009765625</v>
       </c>
       <c r="C32" t="n">
-        <v>0.01759475693602391</v>
+        <v>0.01745414346753853</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>days_quote_to_inception</t>
+          <t>credit_band</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>18007.15185546875</v>
+        <v>17614.12744140625</v>
       </c>
       <c r="C33" t="n">
-        <v>0.01750779582791779</v>
+        <v>0.01739467113184438</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>roof_type</t>
+          <t>wildfire_index</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>17965.05346679688</v>
+        <v>17551.3251953125</v>
       </c>
       <c r="C34" t="n">
-        <v>0.01746686486895952</v>
+        <v>0.01733265134569398</v>
       </c>
     </row>
     <row r="35">
@@ -1094,192 +1094,192 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>17800.65625</v>
+        <v>17445.91064453125</v>
       </c>
       <c r="C35" t="n">
-        <v>0.01730702654863772</v>
+        <v>0.01722855016614645</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>urban_density</t>
+          <t>solar_panels</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>17542.2470703125</v>
+        <v>17272.75927734375</v>
       </c>
       <c r="C36" t="n">
-        <v>0.01705578330959909</v>
+        <v>0.01705755611047863</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>freezing_days</t>
+          <t>branch_id</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>17316.59399414062</v>
+        <v>17229.1025390625</v>
       </c>
       <c r="C37" t="n">
-        <v>0.01683638781511622</v>
+        <v>0.01701444329619831</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>branch_id</t>
+          <t>freezing_days</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>17120.3681640625</v>
+        <v>17064.51293945312</v>
       </c>
       <c r="C38" t="n">
-        <v>0.01664560352025683</v>
+        <v>0.01685190433612488</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>wildfire_index</t>
+          <t>urban_density</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>16955.52563476562</v>
+        <v>16900.47436523438</v>
       </c>
       <c r="C39" t="n">
-        <v>0.01648533223638854</v>
+        <v>0.01668990953615743</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>listed_building</t>
+          <t>renewal_count</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>16786.26416015625</v>
+        <v>16798.67822265625</v>
       </c>
       <c r="C40" t="n">
-        <v>0.01632076454890645</v>
+        <v>0.01658938168267578</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>exposure</t>
+          <t>listed_building</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>16676.05517578125</v>
+        <v>16560.58569335938</v>
       </c>
       <c r="C41" t="n">
-        <v>0.01621361176803768</v>
+        <v>0.01635425557382678</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>renewal_count</t>
+          <t>roof_type</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>16636.55102539062</v>
+        <v>16535.69018554688</v>
       </c>
       <c r="C42" t="n">
-        <v>0.01617520310658219</v>
+        <v>0.01632967024182557</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>marital_status</t>
+          <t>exposure</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>16635.94287109375</v>
+        <v>16506.23095703125</v>
       </c>
       <c r="C43" t="n">
-        <v>0.01617461181700197</v>
+        <v>0.01630057804900865</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>household_size</t>
+          <t>mortgage</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>16424.45776367188</v>
+        <v>16416.30419921875</v>
       </c>
       <c r="C44" t="n">
-        <v>0.01596899139956416</v>
+        <v>0.01621177169835035</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>days_unoccupied</t>
+          <t>household_size</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>16169.28247070312</v>
+        <v>16060.3818359375</v>
       </c>
       <c r="C45" t="n">
-        <v>0.01572089236838566</v>
+        <v>0.01586028381010035</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>mortgage</t>
+          <t>policyholder_age</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>15721.458984375</v>
+        <v>15642.20434570312</v>
       </c>
       <c r="C46" t="n">
-        <v>0.01528548746768239</v>
+        <v>0.01544731643822432</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>policyholder_age</t>
+          <t>Year</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>15570.6201171875</v>
+        <v>15469.93432617188</v>
       </c>
       <c r="C47" t="n">
-        <v>0.01513883151060325</v>
+        <v>0.01527719274940745</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>licence_points</t>
+          <t>days_unoccupied</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>15498.85424804688</v>
+        <v>15422.21875</v>
       </c>
       <c r="C48" t="n">
-        <v>0.01506905577958194</v>
+        <v>0.01523007166673463</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Year</t>
+          <t>licence_points</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>15055.919921875</v>
+        <v>15135.89453125</v>
       </c>
       <c r="C49" t="n">
-        <v>0.01463840445781622</v>
+        <v>0.01494731479224247</v>
       </c>
     </row>
   </sheetData>
@@ -1339,10 +1339,10 @@
         <v>149047</v>
       </c>
       <c r="D2" t="n">
-        <v>107.4767934108967</v>
+        <v>107.7175215714656</v>
       </c>
       <c r="E2" t="n">
-        <v>86.96904754638672</v>
+        <v>88.23249816894531</v>
       </c>
       <c r="F2" t="n">
         <v>191.553809670775</v>
@@ -1359,10 +1359,10 @@
         <v>149047</v>
       </c>
       <c r="D3" t="n">
-        <v>102.5237437279333</v>
+        <v>103.0686088941598</v>
       </c>
       <c r="E3" t="n">
-        <v>88.63224029541016</v>
+        <v>89.84877777099609</v>
       </c>
       <c r="F3" t="n">
         <v>182.4897388072219</v>
@@ -1379,10 +1379,10 @@
         <v>149046</v>
       </c>
       <c r="D4" t="n">
-        <v>101.2626055182601</v>
+        <v>101.3621605269227</v>
       </c>
       <c r="E4" t="n">
-        <v>88.89289093017578</v>
+        <v>89.65425872802734</v>
       </c>
       <c r="F4" t="n">
         <v>182.1870806999182</v>
@@ -1399,10 +1399,10 @@
         <v>149046</v>
       </c>
       <c r="D5" t="n">
-        <v>102.1568385813075</v>
+        <v>101.8815318040999</v>
       </c>
       <c r="E5" t="n">
-        <v>89.24028778076172</v>
+        <v>90.22218322753906</v>
       </c>
       <c r="F5" t="n">
         <v>189.1138007058224</v>

</xml_diff>